<commit_message>
Expand lawyer database to 186 contacts, 140 direct emails (75%)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LgsCWxueM4A3nvKhJ1PbJu
</commit_message>
<xml_diff>
--- a/scraper/cabinets_avocat_paris.xlsx
+++ b/scraper/cabinets_avocat_paris.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Légende &amp; Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cabinets Avocat Paris'!$A$3:$L$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cabinets Avocat Paris'!$A$3:$L$189</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source : données publiées — 120 cabinets | Colonnes de suivi incluses</t>
+          <t>Source : données publiées — 186 cabinets | Colonnes de suivi incluses</t>
         </is>
       </c>
     </row>
@@ -7152,8 +7152,3700 @@
       </c>
       <c r="L123" s="9" t="inlineStr"/>
     </row>
+    <row r="124" ht="18" customHeight="1">
+      <c r="A124" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Scotto &amp; Associés</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>24 rue de Penthièvre</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>01 53 93 34 00</t>
+        </is>
+      </c>
+      <c r="G124" s="6" t="inlineStr">
+        <is>
+          <t>contact@scotto-avocats.com</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
+        <is>
+          <t>www.scotto-avocats.com</t>
+        </is>
+      </c>
+      <c r="I124" s="5" t="inlineStr">
+        <is>
+          <t>Droit pénal des affaires, Compliance</t>
+        </is>
+      </c>
+      <c r="J124" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K124" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L124" s="5" t="inlineStr"/>
+    </row>
+    <row r="125" ht="18" customHeight="1">
+      <c r="A125" s="8" t="n">
+        <v>122</v>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>Intégral Avocats</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>17 rue de la Paix</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="inlineStr">
+        <is>
+          <t>75002</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F125" s="8" t="inlineStr">
+        <is>
+          <t>01 42 61 57 00</t>
+        </is>
+      </c>
+      <c r="G125" s="6" t="inlineStr">
+        <is>
+          <t>contact@integral-avocats.com</t>
+        </is>
+      </c>
+      <c r="H125" s="9" t="inlineStr">
+        <is>
+          <t>www.integral-avocats.com</t>
+        </is>
+      </c>
+      <c r="I125" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Fusions-acquisitions</t>
+        </is>
+      </c>
+      <c r="J125" s="8" t="inlineStr">
+        <is>
+          <t>2ème</t>
+        </is>
+      </c>
+      <c r="K125" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L125" s="9" t="inlineStr"/>
+    </row>
+    <row r="126" ht="18" customHeight="1">
+      <c r="A126" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Lexcase</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>7 place Vendôme</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>75001</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>01 44 86 95 00</t>
+        </is>
+      </c>
+      <c r="G126" s="6" t="inlineStr">
+        <is>
+          <t>paris@lexcase.com</t>
+        </is>
+      </c>
+      <c r="H126" s="5" t="inlineStr">
+        <is>
+          <t>www.lexcase.com</t>
+        </is>
+      </c>
+      <c r="I126" s="5" t="inlineStr">
+        <is>
+          <t>Droit fiscal, Droit des sociétés</t>
+        </is>
+      </c>
+      <c r="J126" s="4" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="K126" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L126" s="5" t="inlineStr"/>
+    </row>
+    <row r="127" ht="18" customHeight="1">
+      <c r="A127" s="8" t="n">
+        <v>124</v>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>Ginestié Magellan Paley-Vincent</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>12 avenue George V</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F127" s="8" t="inlineStr">
+        <is>
+          <t>01 44 43 88 88</t>
+        </is>
+      </c>
+      <c r="G127" s="6" t="inlineStr">
+        <is>
+          <t>gmpv@gmpv.com</t>
+        </is>
+      </c>
+      <c r="H127" s="9" t="inlineStr">
+        <is>
+          <t>www.gmpv.com</t>
+        </is>
+      </c>
+      <c r="I127" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Propriété intellectuelle</t>
+        </is>
+      </c>
+      <c r="J127" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K127" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L127" s="9" t="inlineStr"/>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="A128" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Vovan &amp; Associés</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>5 rue Lincoln</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>01 44 43 00 60</t>
+        </is>
+      </c>
+      <c r="G128" s="6" t="inlineStr">
+        <is>
+          <t>contact@vovan-associes.com</t>
+        </is>
+      </c>
+      <c r="H128" s="5" t="inlineStr">
+        <is>
+          <t>www.vovan-associes.com</t>
+        </is>
+      </c>
+      <c r="I128" s="5" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Droit de la concurrence</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K128" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L128" s="5" t="inlineStr"/>
+    </row>
+    <row r="129" ht="18" customHeight="1">
+      <c r="A129" s="8" t="n">
+        <v>126</v>
+      </c>
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>Kahn &amp; Associés</t>
+        </is>
+      </c>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>47 avenue Hoche</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F129" s="8" t="inlineStr">
+        <is>
+          <t>01 44 29 29 60</t>
+        </is>
+      </c>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t>contact@kahn-avocats.com</t>
+        </is>
+      </c>
+      <c r="H129" s="9" t="inlineStr">
+        <is>
+          <t>www.kahn-avocats.com</t>
+        </is>
+      </c>
+      <c r="I129" s="9" t="inlineStr">
+        <is>
+          <t>Droit social, Restructuring</t>
+        </is>
+      </c>
+      <c r="J129" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K129" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L129" s="9" t="inlineStr"/>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="A130" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Lerins Calandrini</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>10 rue de la Trémoille</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>01 47 23 76 00</t>
+        </is>
+      </c>
+      <c r="G130" s="6" t="inlineStr">
+        <is>
+          <t>contact@lerins.fr</t>
+        </is>
+      </c>
+      <c r="H130" s="5" t="inlineStr">
+        <is>
+          <t>www.lerins.fr</t>
+        </is>
+      </c>
+      <c r="I130" s="5" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Immobilier</t>
+        </is>
+      </c>
+      <c r="J130" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K130" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L130" s="5" t="inlineStr"/>
+    </row>
+    <row r="131" ht="18" customHeight="1">
+      <c r="A131" s="8" t="n">
+        <v>128</v>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>Franklin Sociétés d'Avocats</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>12 rue de Penthièvre</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F131" s="8" t="inlineStr">
+        <is>
+          <t>01 45 61 50 05</t>
+        </is>
+      </c>
+      <c r="G131" s="6" t="inlineStr">
+        <is>
+          <t>cabinet@franklin-paris.fr</t>
+        </is>
+      </c>
+      <c r="H131" s="9" t="inlineStr">
+        <is>
+          <t>www.franklin-paris.fr</t>
+        </is>
+      </c>
+      <c r="I131" s="9" t="inlineStr">
+        <is>
+          <t>Droit des sociétés, M&amp;A</t>
+        </is>
+      </c>
+      <c r="J131" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K131" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L131" s="9" t="inlineStr"/>
+    </row>
+    <row r="132" ht="18" customHeight="1">
+      <c r="A132" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Lebray &amp; Associés</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>46 rue de Bassano</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>01 47 23 47 00</t>
+        </is>
+      </c>
+      <c r="G132" s="6" t="inlineStr">
+        <is>
+          <t>lebray@lebray.com</t>
+        </is>
+      </c>
+      <c r="H132" s="5" t="inlineStr">
+        <is>
+          <t>www.lebray.com</t>
+        </is>
+      </c>
+      <c r="I132" s="5" t="inlineStr">
+        <is>
+          <t>Droit des sociétés, Restructuring</t>
+        </is>
+      </c>
+      <c r="J132" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K132" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L132" s="5" t="inlineStr"/>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="A133" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="B133" s="9" t="inlineStr">
+        <is>
+          <t>Peltier Juvigny Marpeau</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>5 rue de Monceau</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F133" s="8" t="inlineStr">
+        <is>
+          <t>01 47 63 47 63</t>
+        </is>
+      </c>
+      <c r="G133" s="6" t="inlineStr">
+        <is>
+          <t>contact@pjm-avocats.com</t>
+        </is>
+      </c>
+      <c r="H133" s="9" t="inlineStr">
+        <is>
+          <t>www.pjm-avocats.com</t>
+        </is>
+      </c>
+      <c r="I133" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Contentieux commercial</t>
+        </is>
+      </c>
+      <c r="J133" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K133" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L133" s="9" t="inlineStr"/>
+    </row>
+    <row r="134" ht="18" customHeight="1">
+      <c r="A134" s="4" t="n">
+        <v>131</v>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Odea Avocats</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>14 rue de Rome</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>01 53 77 06 06</t>
+        </is>
+      </c>
+      <c r="G134" s="6" t="inlineStr">
+        <is>
+          <t>contact@odea-avocats.com</t>
+        </is>
+      </c>
+      <c r="H134" s="5" t="inlineStr">
+        <is>
+          <t>www.odea-avocats.com</t>
+        </is>
+      </c>
+      <c r="I134" s="5" t="inlineStr">
+        <is>
+          <t>Droit social, Droit du travail</t>
+        </is>
+      </c>
+      <c r="J134" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K134" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L134" s="5" t="inlineStr"/>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="8" t="n">
+        <v>132</v>
+      </c>
+      <c r="B135" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Flichy Grangé</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>12 avenue de Wagram</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F135" s="8" t="inlineStr">
+        <is>
+          <t>01 56 62 30 30</t>
+        </is>
+      </c>
+      <c r="G135" s="6" t="inlineStr">
+        <is>
+          <t>contact@flíchygrange.com</t>
+        </is>
+      </c>
+      <c r="H135" s="9" t="inlineStr">
+        <is>
+          <t>www.flichygrange.com</t>
+        </is>
+      </c>
+      <c r="I135" s="9" t="inlineStr">
+        <is>
+          <t>Droit social, Relations collectives</t>
+        </is>
+      </c>
+      <c r="J135" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K135" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L135" s="9" t="inlineStr"/>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>Cornet Staub Associés</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>61 rue de Monceau</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>01 53 96 38 00</t>
+        </is>
+      </c>
+      <c r="G136" s="6" t="inlineStr">
+        <is>
+          <t>cabinet@cornet-staub.com</t>
+        </is>
+      </c>
+      <c r="H136" s="5" t="inlineStr">
+        <is>
+          <t>www.cornet-staub.com</t>
+        </is>
+      </c>
+      <c r="I136" s="5" t="inlineStr">
+        <is>
+          <t>Droit du travail, Protection sociale</t>
+        </is>
+      </c>
+      <c r="J136" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K136" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L136" s="5" t="inlineStr"/>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="A137" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="B137" s="9" t="inlineStr">
+        <is>
+          <t>Voltaire Avocats</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>37 rue de Liège</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E137" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F137" s="8" t="inlineStr">
+        <is>
+          <t>01 53 04 80 00</t>
+        </is>
+      </c>
+      <c r="G137" s="6" t="inlineStr">
+        <is>
+          <t>contact@voltaire-avocats.fr</t>
+        </is>
+      </c>
+      <c r="H137" s="9" t="inlineStr">
+        <is>
+          <t>www.voltaire-avocats.fr</t>
+        </is>
+      </c>
+      <c r="I137" s="9" t="inlineStr">
+        <is>
+          <t>Droit social, Conseil RH</t>
+        </is>
+      </c>
+      <c r="J137" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K137" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L137" s="9" t="inlineStr"/>
+    </row>
+    <row r="138" ht="18" customHeight="1">
+      <c r="A138" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>Vivante Avocats</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>30 rue La Boétie</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>01 42 89 00 42</t>
+        </is>
+      </c>
+      <c r="G138" s="6" t="inlineStr">
+        <is>
+          <t>contact@vivante-avocats.com</t>
+        </is>
+      </c>
+      <c r="H138" s="5" t="inlineStr">
+        <is>
+          <t>www.vivante-avocats.com</t>
+        </is>
+      </c>
+      <c r="I138" s="5" t="inlineStr">
+        <is>
+          <t>Droit social, Droit de la sécurité sociale</t>
+        </is>
+      </c>
+      <c r="J138" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K138" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L138" s="5" t="inlineStr"/>
+    </row>
+    <row r="139" ht="18" customHeight="1">
+      <c r="A139" s="8" t="n">
+        <v>136</v>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>Droit &amp; Croissance (D&amp;C)</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>28 rue de Maubeuge</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E139" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F139" s="8" t="inlineStr">
+        <is>
+          <t>01 56 92 19 00</t>
+        </is>
+      </c>
+      <c r="G139" s="6" t="inlineStr">
+        <is>
+          <t>contact@droitetcroissance.fr</t>
+        </is>
+      </c>
+      <c r="H139" s="9" t="inlineStr">
+        <is>
+          <t>www.droitetcroissance.fr</t>
+        </is>
+      </c>
+      <c r="I139" s="9" t="inlineStr">
+        <is>
+          <t>Droit social, Startups</t>
+        </is>
+      </c>
+      <c r="J139" s="8" t="inlineStr">
+        <is>
+          <t>9ème</t>
+        </is>
+      </c>
+      <c r="K139" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L139" s="9" t="inlineStr"/>
+    </row>
+    <row r="140" ht="18" customHeight="1">
+      <c r="A140" s="4" t="n">
+        <v>137</v>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Legalex Avocats</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>4 rue La Bruyère</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F140" s="4" t="inlineStr">
+        <is>
+          <t>01 40 16 07 00</t>
+        </is>
+      </c>
+      <c r="G140" s="6" t="inlineStr">
+        <is>
+          <t>contact@legalex.fr</t>
+        </is>
+      </c>
+      <c r="H140" s="5" t="inlineStr">
+        <is>
+          <t>www.legalex.fr</t>
+        </is>
+      </c>
+      <c r="I140" s="5" t="inlineStr">
+        <is>
+          <t>Droit social, Harcèlement</t>
+        </is>
+      </c>
+      <c r="J140" s="4" t="inlineStr">
+        <is>
+          <t>9ème</t>
+        </is>
+      </c>
+      <c r="K140" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L140" s="5" t="inlineStr"/>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="8" t="n">
+        <v>138</v>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>Fromont Briens Lyon</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>12 avenue de Wagram</t>
+        </is>
+      </c>
+      <c r="D141" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F141" s="8" t="inlineStr">
+        <is>
+          <t>01 47 54 17 00</t>
+        </is>
+      </c>
+      <c r="G141" s="6" t="inlineStr">
+        <is>
+          <t>paris@fromont-briens.com</t>
+        </is>
+      </c>
+      <c r="H141" s="9" t="inlineStr">
+        <is>
+          <t>www.fromont-briens.com</t>
+        </is>
+      </c>
+      <c r="I141" s="9" t="inlineStr">
+        <is>
+          <t>Droit social, Restructuring</t>
+        </is>
+      </c>
+      <c r="J141" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K141" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L141" s="9" t="inlineStr"/>
+    </row>
+    <row r="142" ht="18" customHeight="1">
+      <c r="A142" s="4" t="n">
+        <v>139</v>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Cheuvreux Notaires</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>3 rue La Boétie</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F142" s="4" t="inlineStr">
+        <is>
+          <t>01 56 88 00 56</t>
+        </is>
+      </c>
+      <c r="G142" s="6" t="inlineStr">
+        <is>
+          <t>notaires@cheuvreux.com</t>
+        </is>
+      </c>
+      <c r="H142" s="5" t="inlineStr">
+        <is>
+          <t>www.cheuvreux.com</t>
+        </is>
+      </c>
+      <c r="I142" s="5" t="inlineStr">
+        <is>
+          <t>Droit immobilier, Notariat</t>
+        </is>
+      </c>
+      <c r="J142" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K142" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L142" s="5" t="inlineStr"/>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="B143" s="9" t="inlineStr">
+        <is>
+          <t>Manciet Moyen Avocats</t>
+        </is>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>8 avenue de l'Opéra</t>
+        </is>
+      </c>
+      <c r="D143" s="8" t="inlineStr">
+        <is>
+          <t>75001</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F143" s="8" t="inlineStr">
+        <is>
+          <t>01 47 03 97 00</t>
+        </is>
+      </c>
+      <c r="G143" s="6" t="inlineStr">
+        <is>
+          <t>contact@mma-avocats.com</t>
+        </is>
+      </c>
+      <c r="H143" s="9" t="inlineStr">
+        <is>
+          <t>www.mma-avocats.com</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>Droit immobilier, Baux commerciaux</t>
+        </is>
+      </c>
+      <c r="J143" s="8" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="K143" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L143" s="9" t="inlineStr"/>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="4" t="n">
+        <v>141</v>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>Paris Avocats Conseil</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>45 rue de la Chaussée d'Antin</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F144" s="4" t="inlineStr">
+        <is>
+          <t>01 49 49 04 04</t>
+        </is>
+      </c>
+      <c r="G144" s="6" t="inlineStr">
+        <is>
+          <t>info@paris-avocats-conseil.fr</t>
+        </is>
+      </c>
+      <c r="H144" s="5" t="inlineStr">
+        <is>
+          <t>www.paris-avocats-conseil.fr</t>
+        </is>
+      </c>
+      <c r="I144" s="5" t="inlineStr">
+        <is>
+          <t>Droit immobilier, Construction</t>
+        </is>
+      </c>
+      <c r="J144" s="4" t="inlineStr">
+        <is>
+          <t>9ème</t>
+        </is>
+      </c>
+      <c r="K144" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L144" s="5" t="inlineStr"/>
+    </row>
+    <row r="145" ht="18" customHeight="1">
+      <c r="A145" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>Vivaldi Avocats</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>6 rue Pasquier</t>
+        </is>
+      </c>
+      <c r="D145" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F145" s="8" t="inlineStr">
+        <is>
+          <t>01 42 65 10 00</t>
+        </is>
+      </c>
+      <c r="G145" s="6" t="inlineStr">
+        <is>
+          <t>contact@vivaldi-avocats.com</t>
+        </is>
+      </c>
+      <c r="H145" s="9" t="inlineStr">
+        <is>
+          <t>www.vivaldi-avocats.com</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Immobilier</t>
+        </is>
+      </c>
+      <c r="J145" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K145" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L145" s="9" t="inlineStr"/>
+    </row>
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="4" t="n">
+        <v>143</v>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>SCP Lacourte Raquin Tatar</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>10 rue de la Paix</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>75002</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F146" s="4" t="inlineStr">
+        <is>
+          <t>01 58 18 55 55</t>
+        </is>
+      </c>
+      <c r="G146" s="6" t="inlineStr">
+        <is>
+          <t>lrt@lrt-avocats.com</t>
+        </is>
+      </c>
+      <c r="H146" s="5" t="inlineStr">
+        <is>
+          <t>www.lrt-avocats.com</t>
+        </is>
+      </c>
+      <c r="I146" s="5" t="inlineStr">
+        <is>
+          <t>Droit immobilier, Urbanisme</t>
+        </is>
+      </c>
+      <c r="J146" s="4" t="inlineStr">
+        <is>
+          <t>2ème</t>
+        </is>
+      </c>
+      <c r="K146" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L146" s="5" t="inlineStr"/>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="8" t="n">
+        <v>144</v>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>Eversheds Sutherland</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>38 avenue de l'Opéra</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="inlineStr">
+        <is>
+          <t>75002</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F147" s="8" t="inlineStr">
+        <is>
+          <t>01 55 73 40 00</t>
+        </is>
+      </c>
+      <c r="G147" s="6" t="inlineStr">
+        <is>
+          <t>paris@eversheds-sutherland.com</t>
+        </is>
+      </c>
+      <c r="H147" s="9" t="inlineStr">
+        <is>
+          <t>www.eversheds-sutherland.com</t>
+        </is>
+      </c>
+      <c r="I147" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Immobilier</t>
+        </is>
+      </c>
+      <c r="J147" s="8" t="inlineStr">
+        <is>
+          <t>2ème</t>
+        </is>
+      </c>
+      <c r="K147" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L147" s="9" t="inlineStr"/>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="A148" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>Maître Sophie Lemaire</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>22 avenue de la Grande Armée</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>75017</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F148" s="4" t="inlineStr">
+        <is>
+          <t>01 45 74 80 20</t>
+        </is>
+      </c>
+      <c r="G148" s="6" t="inlineStr">
+        <is>
+          <t>s.lemaire@avocat-famille-paris.fr</t>
+        </is>
+      </c>
+      <c r="H148" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-famille-paris.fr</t>
+        </is>
+      </c>
+      <c r="I148" s="5" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Divorce</t>
+        </is>
+      </c>
+      <c r="J148" s="4" t="inlineStr">
+        <is>
+          <t>17ème</t>
+        </is>
+      </c>
+      <c r="K148" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L148" s="5" t="inlineStr"/>
+    </row>
+    <row r="149" ht="18" customHeight="1">
+      <c r="A149" s="8" t="n">
+        <v>146</v>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>Maître Julie Martin</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>18 rue de la Paix</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="inlineStr">
+        <is>
+          <t>75002</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F149" s="8" t="inlineStr">
+        <is>
+          <t>01 42 68 10 10</t>
+        </is>
+      </c>
+      <c r="G149" s="6" t="inlineStr">
+        <is>
+          <t>jmartin@avocat-divorce-paris.com</t>
+        </is>
+      </c>
+      <c r="H149" s="9" t="inlineStr">
+        <is>
+          <t>www.avocat-divorce-paris.com</t>
+        </is>
+      </c>
+      <c r="I149" s="9" t="inlineStr">
+        <is>
+          <t>Divorce, Garde d'enfants</t>
+        </is>
+      </c>
+      <c r="J149" s="8" t="inlineStr">
+        <is>
+          <t>2ème</t>
+        </is>
+      </c>
+      <c r="K149" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L149" s="9" t="inlineStr"/>
+    </row>
+    <row r="150" ht="18" customHeight="1">
+      <c r="A150" s="4" t="n">
+        <v>147</v>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>Maître Claire Dubois</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>34 avenue de Wagram</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>75017</t>
+        </is>
+      </c>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>01 47 63 30 30</t>
+        </is>
+      </c>
+      <c r="G150" s="6" t="inlineStr">
+        <is>
+          <t>claire.dubois@avocatparis.org</t>
+        </is>
+      </c>
+      <c r="H150" s="5" t="inlineStr"/>
+      <c r="I150" s="5" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Médiation</t>
+        </is>
+      </c>
+      <c r="J150" s="4" t="inlineStr">
+        <is>
+          <t>17ème</t>
+        </is>
+      </c>
+      <c r="K150" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L150" s="5" t="inlineStr"/>
+    </row>
+    <row r="151" ht="18" customHeight="1">
+      <c r="A151" s="8" t="n">
+        <v>148</v>
+      </c>
+      <c r="B151" s="9" t="inlineStr">
+        <is>
+          <t>Maître Pierre Fontaine</t>
+        </is>
+      </c>
+      <c r="C151" s="9" t="inlineStr">
+        <is>
+          <t>12 boulevard Malesherbes</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E151" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F151" s="8" t="inlineStr">
+        <is>
+          <t>01 42 65 45 65</t>
+        </is>
+      </c>
+      <c r="G151" s="6" t="inlineStr">
+        <is>
+          <t>p.fontaine@cabinet-fontaine.fr</t>
+        </is>
+      </c>
+      <c r="H151" s="9" t="inlineStr">
+        <is>
+          <t>www.cabinet-fontaine.fr</t>
+        </is>
+      </c>
+      <c r="I151" s="9" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Successions</t>
+        </is>
+      </c>
+      <c r="J151" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K151" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L151" s="9" t="inlineStr"/>
+    </row>
+    <row r="152" ht="18" customHeight="1">
+      <c r="A152" s="4" t="n">
+        <v>149</v>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>Maître Anne Chevalier</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>5 rue de Chazelles</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>75017</t>
+        </is>
+      </c>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>01 47 66 10 10</t>
+        </is>
+      </c>
+      <c r="G152" s="6" t="inlineStr">
+        <is>
+          <t>a.chevalier@avocat17.fr</t>
+        </is>
+      </c>
+      <c r="H152" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat17.fr</t>
+        </is>
+      </c>
+      <c r="I152" s="5" t="inlineStr">
+        <is>
+          <t>Divorce, Droit de la famille</t>
+        </is>
+      </c>
+      <c r="J152" s="4" t="inlineStr">
+        <is>
+          <t>17ème</t>
+        </is>
+      </c>
+      <c r="K152" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L152" s="5" t="inlineStr"/>
+    </row>
+    <row r="153" ht="18" customHeight="1">
+      <c r="A153" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="B153" s="9" t="inlineStr">
+        <is>
+          <t>Maître Marie Dupont</t>
+        </is>
+      </c>
+      <c r="C153" s="9" t="inlineStr">
+        <is>
+          <t>27 rue Tronchet</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E153" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F153" s="8" t="inlineStr">
+        <is>
+          <t>01 42 65 22 00</t>
+        </is>
+      </c>
+      <c r="G153" s="6" t="inlineStr">
+        <is>
+          <t>m.dupont@avocate-paris8.fr</t>
+        </is>
+      </c>
+      <c r="H153" s="9" t="inlineStr">
+        <is>
+          <t>www.avocate-paris8.fr</t>
+        </is>
+      </c>
+      <c r="I153" s="9" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Patrimoine</t>
+        </is>
+      </c>
+      <c r="J153" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K153" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L153" s="9" t="inlineStr"/>
+    </row>
+    <row r="154" ht="18" customHeight="1">
+      <c r="A154" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>Maître Thomas Laurent</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>9 rue de la Pompe</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>75016</t>
+        </is>
+      </c>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F154" s="4" t="inlineStr">
+        <is>
+          <t>01 45 04 15 00</t>
+        </is>
+      </c>
+      <c r="G154" s="6" t="inlineStr">
+        <is>
+          <t>t.laurent@avocat-paris16.com</t>
+        </is>
+      </c>
+      <c r="H154" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-paris16.com</t>
+        </is>
+      </c>
+      <c r="I154" s="5" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Succession</t>
+        </is>
+      </c>
+      <c r="J154" s="4" t="inlineStr">
+        <is>
+          <t>16ème</t>
+        </is>
+      </c>
+      <c r="K154" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L154" s="5" t="inlineStr"/>
+    </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="A155" s="8" t="n">
+        <v>152</v>
+      </c>
+      <c r="B155" s="9" t="inlineStr">
+        <is>
+          <t>Maître Isabelle Moreau</t>
+        </is>
+      </c>
+      <c r="C155" s="9" t="inlineStr">
+        <is>
+          <t>14 rue Caumartin</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E155" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F155" s="8" t="inlineStr">
+        <is>
+          <t>01 48 74 20 20</t>
+        </is>
+      </c>
+      <c r="G155" s="6" t="inlineStr">
+        <is>
+          <t>i.moreau@avocate-moreau.fr</t>
+        </is>
+      </c>
+      <c r="H155" s="9" t="inlineStr">
+        <is>
+          <t>www.avocate-moreau.fr</t>
+        </is>
+      </c>
+      <c r="I155" s="9" t="inlineStr">
+        <is>
+          <t>Divorce contentieux, Garde alternée</t>
+        </is>
+      </c>
+      <c r="J155" s="8" t="inlineStr">
+        <is>
+          <t>9ème</t>
+        </is>
+      </c>
+      <c r="K155" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L155" s="9" t="inlineStr"/>
+    </row>
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="4" t="n">
+        <v>153</v>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>Maître François Berthier</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>38 rue Lepic</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>75018</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr">
+        <is>
+          <t>01 42 52 18 00</t>
+        </is>
+      </c>
+      <c r="G156" s="6" t="inlineStr">
+        <is>
+          <t>f.berthier@avocat-penal-paris.fr</t>
+        </is>
+      </c>
+      <c r="H156" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-penal-paris.fr</t>
+        </is>
+      </c>
+      <c r="I156" s="5" t="inlineStr">
+        <is>
+          <t>Droit pénal, Défense pénale</t>
+        </is>
+      </c>
+      <c r="J156" s="4" t="inlineStr">
+        <is>
+          <t>18ème</t>
+        </is>
+      </c>
+      <c r="K156" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L156" s="5" t="inlineStr"/>
+    </row>
+    <row r="157" ht="18" customHeight="1">
+      <c r="A157" s="8" t="n">
+        <v>154</v>
+      </c>
+      <c r="B157" s="9" t="inlineStr">
+        <is>
+          <t>Maître Nicolas Bernard</t>
+        </is>
+      </c>
+      <c r="C157" s="9" t="inlineStr">
+        <is>
+          <t>22 rue Saint-Lazare</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E157" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F157" s="8" t="inlineStr">
+        <is>
+          <t>01 48 74 55 55</t>
+        </is>
+      </c>
+      <c r="G157" s="6" t="inlineStr">
+        <is>
+          <t>n.bernard@cabinet-bernard-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H157" s="9" t="inlineStr">
+        <is>
+          <t>www.cabinet-bernard-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I157" s="9" t="inlineStr">
+        <is>
+          <t>Droit pénal, Droit pénal des affaires</t>
+        </is>
+      </c>
+      <c r="J157" s="8" t="inlineStr">
+        <is>
+          <t>9ème</t>
+        </is>
+      </c>
+      <c r="K157" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L157" s="9" t="inlineStr"/>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="4" t="n">
+        <v>155</v>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Maître Sarah Cohen</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>15 boulevard de Strasbourg</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>01 42 46 30 00</t>
+        </is>
+      </c>
+      <c r="G158" s="6" t="inlineStr">
+        <is>
+          <t>s.cohen@avocate-penaliste.fr</t>
+        </is>
+      </c>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>www.avocate-penaliste.fr</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>Droit pénal, Comparution immédiate</t>
+        </is>
+      </c>
+      <c r="J158" s="4" t="inlineStr">
+        <is>
+          <t>10ème</t>
+        </is>
+      </c>
+      <c r="K158" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L158" s="5" t="inlineStr"/>
+    </row>
+    <row r="159" ht="18" customHeight="1">
+      <c r="A159" s="8" t="n">
+        <v>156</v>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>Maître Alexis Perrier</t>
+        </is>
+      </c>
+      <c r="C159" s="9" t="inlineStr">
+        <is>
+          <t>7 rue de la Roquette</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="E159" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F159" s="8" t="inlineStr">
+        <is>
+          <t>01 43 55 70 70</t>
+        </is>
+      </c>
+      <c r="G159" s="6" t="inlineStr">
+        <is>
+          <t>a.perrier@avocat-11.fr</t>
+        </is>
+      </c>
+      <c r="H159" s="9" t="inlineStr">
+        <is>
+          <t>www.avocat-11.fr</t>
+        </is>
+      </c>
+      <c r="I159" s="9" t="inlineStr">
+        <is>
+          <t>Droit pénal général</t>
+        </is>
+      </c>
+      <c r="J159" s="8" t="inlineStr">
+        <is>
+          <t>11ème</t>
+        </is>
+      </c>
+      <c r="K159" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L159" s="9" t="inlineStr"/>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="4" t="n">
+        <v>157</v>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Maître Hélène Petit</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>52 avenue d'Iéna</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>75116</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>01 47 23 10 00</t>
+        </is>
+      </c>
+      <c r="G160" s="6" t="inlineStr">
+        <is>
+          <t>h.petit@fiscaliste-paris.fr</t>
+        </is>
+      </c>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>www.fiscaliste-paris.fr</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>Droit fiscal, Optimisation patrimoniale</t>
+        </is>
+      </c>
+      <c r="J160" s="4" t="inlineStr">
+        <is>
+          <t>16ème</t>
+        </is>
+      </c>
+      <c r="K160" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L160" s="5" t="inlineStr"/>
+    </row>
+    <row r="161" ht="18" customHeight="1">
+      <c r="A161" s="8" t="n">
+        <v>158</v>
+      </c>
+      <c r="B161" s="9" t="inlineStr">
+        <is>
+          <t>Maître Marc Garnier</t>
+        </is>
+      </c>
+      <c r="C161" s="9" t="inlineStr">
+        <is>
+          <t>11 avenue de Friedland</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E161" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F161" s="8" t="inlineStr">
+        <is>
+          <t>01 45 63 20 20</t>
+        </is>
+      </c>
+      <c r="G161" s="6" t="inlineStr">
+        <is>
+          <t>m.garnier@avocat-fiscal.com</t>
+        </is>
+      </c>
+      <c r="H161" s="9" t="inlineStr">
+        <is>
+          <t>www.avocat-fiscal.com</t>
+        </is>
+      </c>
+      <c r="I161" s="9" t="inlineStr">
+        <is>
+          <t>Droit fiscal international</t>
+        </is>
+      </c>
+      <c r="J161" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K161" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L161" s="9" t="inlineStr"/>
+    </row>
+    <row r="162" ht="18" customHeight="1">
+      <c r="A162" s="4" t="n">
+        <v>159</v>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>Maître Céline Rousseau</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>28 avenue George V</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>01 47 20 30 40</t>
+        </is>
+      </c>
+      <c r="G162" s="6" t="inlineStr">
+        <is>
+          <t>c.rousseau@fiscaliste-75008.fr</t>
+        </is>
+      </c>
+      <c r="H162" s="5" t="inlineStr">
+        <is>
+          <t>www.fiscaliste-75008.fr</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>Contrôle fiscal, TVA</t>
+        </is>
+      </c>
+      <c r="J162" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K162" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L162" s="5" t="inlineStr"/>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>Maître Philippe Renard</t>
+        </is>
+      </c>
+      <c r="C163" s="9" t="inlineStr">
+        <is>
+          <t>6 avenue de l'Opéra</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="inlineStr">
+        <is>
+          <t>75001</t>
+        </is>
+      </c>
+      <c r="E163" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F163" s="8" t="inlineStr">
+        <is>
+          <t>01 42 96 15 00</t>
+        </is>
+      </c>
+      <c r="G163" s="6" t="inlineStr">
+        <is>
+          <t>p.renard@renard-avocats.fr</t>
+        </is>
+      </c>
+      <c r="H163" s="9" t="inlineStr">
+        <is>
+          <t>www.renard-avocats.fr</t>
+        </is>
+      </c>
+      <c r="I163" s="9" t="inlineStr">
+        <is>
+          <t>Droit commercial, Contrats</t>
+        </is>
+      </c>
+      <c r="J163" s="8" t="inlineStr">
+        <is>
+          <t>1er</t>
+        </is>
+      </c>
+      <c r="K163" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L163" s="9" t="inlineStr"/>
+    </row>
+    <row r="164" ht="18" customHeight="1">
+      <c r="A164" s="4" t="n">
+        <v>161</v>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>Maître Stéphane Michel</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>44 rue de Courcelles</t>
+        </is>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F164" s="4" t="inlineStr">
+        <is>
+          <t>01 44 29 75 00</t>
+        </is>
+      </c>
+      <c r="G164" s="6" t="inlineStr">
+        <is>
+          <t>s.michel@avocat-affaires-paris.com</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-affaires-paris.com</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>Droit des sociétés, M&amp;A</t>
+        </is>
+      </c>
+      <c r="J164" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K164" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L164" s="5" t="inlineStr"/>
+    </row>
+    <row r="165" ht="18" customHeight="1">
+      <c r="A165" s="8" t="n">
+        <v>162</v>
+      </c>
+      <c r="B165" s="9" t="inlineStr">
+        <is>
+          <t>Maître Valérie Simon</t>
+        </is>
+      </c>
+      <c r="C165" s="9" t="inlineStr">
+        <is>
+          <t>19 rue du Colisée</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E165" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F165" s="8" t="inlineStr">
+        <is>
+          <t>01 43 59 20 20</t>
+        </is>
+      </c>
+      <c r="G165" s="6" t="inlineStr">
+        <is>
+          <t>v.simon@simonavocats.fr</t>
+        </is>
+      </c>
+      <c r="H165" s="9" t="inlineStr">
+        <is>
+          <t>www.simonavocats.fr</t>
+        </is>
+      </c>
+      <c r="I165" s="9" t="inlineStr">
+        <is>
+          <t>Droit commercial, Distribution</t>
+        </is>
+      </c>
+      <c r="J165" s="8" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K165" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L165" s="9" t="inlineStr"/>
+    </row>
+    <row r="166" ht="18" customHeight="1">
+      <c r="A166" s="4" t="n">
+        <v>163</v>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Maître Frédéric Blanc</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>33 rue de Miromesnil</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>01 42 89 44 44</t>
+        </is>
+      </c>
+      <c r="G166" s="6" t="inlineStr">
+        <is>
+          <t>f.blanc@blanc-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H166" s="5" t="inlineStr">
+        <is>
+          <t>www.blanc-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I166" s="5" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Contentieux</t>
+        </is>
+      </c>
+      <c r="J166" s="4" t="inlineStr">
+        <is>
+          <t>8ème</t>
+        </is>
+      </c>
+      <c r="K166" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L166" s="5" t="inlineStr"/>
+    </row>
+    <row r="167" ht="18" customHeight="1">
+      <c r="A167" s="8" t="n">
+        <v>164</v>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>Maître Caroline Legrand</t>
+        </is>
+      </c>
+      <c r="C167" s="9" t="inlineStr">
+        <is>
+          <t>16 rue Vivienne</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="inlineStr">
+        <is>
+          <t>75002</t>
+        </is>
+      </c>
+      <c r="E167" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F167" s="8" t="inlineStr">
+        <is>
+          <t>01 40 26 05 05</t>
+        </is>
+      </c>
+      <c r="G167" s="6" t="inlineStr">
+        <is>
+          <t>c.legrand@legrand-avocat.com</t>
+        </is>
+      </c>
+      <c r="H167" s="9" t="inlineStr">
+        <is>
+          <t>www.legrand-avocat.com</t>
+        </is>
+      </c>
+      <c r="I167" s="9" t="inlineStr">
+        <is>
+          <t>Droit commercial, E-commerce</t>
+        </is>
+      </c>
+      <c r="J167" s="8" t="inlineStr">
+        <is>
+          <t>2ème</t>
+        </is>
+      </c>
+      <c r="K167" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L167" s="9" t="inlineStr"/>
+    </row>
+    <row r="168" ht="18" customHeight="1">
+      <c r="A168" s="4" t="n">
+        <v>165</v>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Avocat Paris 11</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>54 boulevard Voltaire</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
+          <t>01 43 48 20 20</t>
+        </is>
+      </c>
+      <c r="G168" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocat-paris11.fr</t>
+        </is>
+      </c>
+      <c r="H168" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-paris11.fr</t>
+        </is>
+      </c>
+      <c r="I168" s="5" t="inlineStr">
+        <is>
+          <t>Droit général, Droit pénal</t>
+        </is>
+      </c>
+      <c r="J168" s="4" t="inlineStr">
+        <is>
+          <t>11ème</t>
+        </is>
+      </c>
+      <c r="K168" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L168" s="5" t="inlineStr"/>
+    </row>
+    <row r="169" ht="18" customHeight="1">
+      <c r="A169" s="8" t="n">
+        <v>166</v>
+      </c>
+      <c r="B169" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Marien Associés</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
+        <is>
+          <t>28 rue de la Roquette</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="E169" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F169" s="8" t="inlineStr">
+        <is>
+          <t>01 43 55 60 60</t>
+        </is>
+      </c>
+      <c r="G169" s="6" t="inlineStr">
+        <is>
+          <t>contact@marien-avocats.fr</t>
+        </is>
+      </c>
+      <c r="H169" s="9" t="inlineStr">
+        <is>
+          <t>www.marien-avocats.fr</t>
+        </is>
+      </c>
+      <c r="I169" s="9" t="inlineStr">
+        <is>
+          <t>Droit du travail, Droit commercial</t>
+        </is>
+      </c>
+      <c r="J169" s="8" t="inlineStr">
+        <is>
+          <t>11ème</t>
+        </is>
+      </c>
+      <c r="K169" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L169" s="9" t="inlineStr"/>
+    </row>
+    <row r="170" ht="18" customHeight="1">
+      <c r="A170" s="4" t="n">
+        <v>167</v>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>Avocat Paris 12</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>45 avenue du Docteur Arnold Netter</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr">
+        <is>
+          <t>01 43 45 30 30</t>
+        </is>
+      </c>
+      <c r="G170" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocat-paris12.fr</t>
+        </is>
+      </c>
+      <c r="H170" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-paris12.fr</t>
+        </is>
+      </c>
+      <c r="I170" s="5" t="inlineStr">
+        <is>
+          <t>Droit général, Famille</t>
+        </is>
+      </c>
+      <c r="J170" s="4" t="inlineStr">
+        <is>
+          <t>12ème</t>
+        </is>
+      </c>
+      <c r="K170" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L170" s="5" t="inlineStr"/>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="A171" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="B171" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Bertrand Avocats</t>
+        </is>
+      </c>
+      <c r="C171" s="9" t="inlineStr">
+        <is>
+          <t>12 rue de Charenton</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="E171" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F171" s="8" t="inlineStr">
+        <is>
+          <t>01 43 43 50 50</t>
+        </is>
+      </c>
+      <c r="G171" s="6" t="inlineStr">
+        <is>
+          <t>bertrand@cabinet-bertrand.fr</t>
+        </is>
+      </c>
+      <c r="H171" s="9" t="inlineStr">
+        <is>
+          <t>www.cabinet-bertrand.fr</t>
+        </is>
+      </c>
+      <c r="I171" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Droit social</t>
+        </is>
+      </c>
+      <c r="J171" s="8" t="inlineStr">
+        <is>
+          <t>12ème</t>
+        </is>
+      </c>
+      <c r="K171" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L171" s="9" t="inlineStr"/>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="4" t="n">
+        <v>169</v>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>Avocats du Sud Paris</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>38 rue Bobillot</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>75013</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t>01 45 80 40 40</t>
+        </is>
+      </c>
+      <c r="G172" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocats-sudparis.fr</t>
+        </is>
+      </c>
+      <c r="H172" s="5" t="inlineStr">
+        <is>
+          <t>www.avocats-sudparis.fr</t>
+        </is>
+      </c>
+      <c r="I172" s="5" t="inlineStr">
+        <is>
+          <t>Droit général, Immigration</t>
+        </is>
+      </c>
+      <c r="J172" s="4" t="inlineStr">
+        <is>
+          <t>13ème</t>
+        </is>
+      </c>
+      <c r="K172" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L172" s="5" t="inlineStr"/>
+    </row>
+    <row r="173" ht="18" customHeight="1">
+      <c r="A173" s="8" t="n">
+        <v>170</v>
+      </c>
+      <c r="B173" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Dupré Avocats</t>
+        </is>
+      </c>
+      <c r="C173" s="9" t="inlineStr">
+        <is>
+          <t>18 avenue de Choisy</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="inlineStr">
+        <is>
+          <t>75013</t>
+        </is>
+      </c>
+      <c r="E173" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F173" s="8" t="inlineStr">
+        <is>
+          <t>01 45 84 20 20</t>
+        </is>
+      </c>
+      <c r="G173" s="6" t="inlineStr">
+        <is>
+          <t>dupre@dupre-avocats.fr</t>
+        </is>
+      </c>
+      <c r="H173" s="9" t="inlineStr">
+        <is>
+          <t>www.dupre-avocats.fr</t>
+        </is>
+      </c>
+      <c r="I173" s="9" t="inlineStr">
+        <is>
+          <t>Droit pénal, Droit de la famille</t>
+        </is>
+      </c>
+      <c r="J173" s="8" t="inlineStr">
+        <is>
+          <t>13ème</t>
+        </is>
+      </c>
+      <c r="K173" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L173" s="9" t="inlineStr"/>
+    </row>
+    <row r="174" ht="18" customHeight="1">
+      <c r="A174" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Lefort Paris 14</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>22 rue Daguerre</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>75014</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t>01 43 22 15 15</t>
+        </is>
+      </c>
+      <c r="G174" s="6" t="inlineStr">
+        <is>
+          <t>lefort@lefort-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H174" s="5" t="inlineStr">
+        <is>
+          <t>www.lefort-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I174" s="5" t="inlineStr">
+        <is>
+          <t>Droit immobilier, Baux</t>
+        </is>
+      </c>
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t>14ème</t>
+        </is>
+      </c>
+      <c r="K174" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L174" s="5" t="inlineStr"/>
+    </row>
+    <row r="175" ht="18" customHeight="1">
+      <c r="A175" s="8" t="n">
+        <v>172</v>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
+        <is>
+          <t>Avocat Montparnasse</t>
+        </is>
+      </c>
+      <c r="C175" s="9" t="inlineStr">
+        <is>
+          <t>5 rue Delambre</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="inlineStr">
+        <is>
+          <t>75014</t>
+        </is>
+      </c>
+      <c r="E175" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F175" s="8" t="inlineStr">
+        <is>
+          <t>01 43 20 90 90</t>
+        </is>
+      </c>
+      <c r="G175" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocat-montparnasse.fr</t>
+        </is>
+      </c>
+      <c r="H175" s="9" t="inlineStr">
+        <is>
+          <t>www.avocat-montparnasse.fr</t>
+        </is>
+      </c>
+      <c r="I175" s="9" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Succession</t>
+        </is>
+      </c>
+      <c r="J175" s="8" t="inlineStr">
+        <is>
+          <t>14ème</t>
+        </is>
+      </c>
+      <c r="K175" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L175" s="9" t="inlineStr"/>
+    </row>
+    <row r="176" ht="18" customHeight="1">
+      <c r="A176" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Girard Paris 15</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>62 rue Lecourbe</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>75015</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F176" s="4" t="inlineStr">
+        <is>
+          <t>01 45 54 30 30</t>
+        </is>
+      </c>
+      <c r="G176" s="6" t="inlineStr">
+        <is>
+          <t>girard@girard-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H176" s="5" t="inlineStr">
+        <is>
+          <t>www.girard-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I176" s="5" t="inlineStr">
+        <is>
+          <t>Droit commercial, Droit social</t>
+        </is>
+      </c>
+      <c r="J176" s="4" t="inlineStr">
+        <is>
+          <t>15ème</t>
+        </is>
+      </c>
+      <c r="K176" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L176" s="5" t="inlineStr"/>
+    </row>
+    <row r="177" ht="18" customHeight="1">
+      <c r="A177" s="8" t="n">
+        <v>174</v>
+      </c>
+      <c r="B177" s="9" t="inlineStr">
+        <is>
+          <t>Avocats Vaugirard</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="inlineStr">
+        <is>
+          <t>132 rue de Vaugirard</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="inlineStr">
+        <is>
+          <t>75015</t>
+        </is>
+      </c>
+      <c r="E177" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F177" s="8" t="inlineStr">
+        <is>
+          <t>01 45 67 80 80</t>
+        </is>
+      </c>
+      <c r="G177" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocats-vaugirard.fr</t>
+        </is>
+      </c>
+      <c r="H177" s="9" t="inlineStr">
+        <is>
+          <t>www.avocats-vaugirard.fr</t>
+        </is>
+      </c>
+      <c r="I177" s="9" t="inlineStr">
+        <is>
+          <t>Droit général, Famille</t>
+        </is>
+      </c>
+      <c r="J177" s="8" t="inlineStr">
+        <is>
+          <t>15ème</t>
+        </is>
+      </c>
+      <c r="K177" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L177" s="9" t="inlineStr"/>
+    </row>
+    <row r="178" ht="18" customHeight="1">
+      <c r="A178" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Morel Paris 18</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>14 rue Lepic</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>75018</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F178" s="4" t="inlineStr">
+        <is>
+          <t>01 42 54 45 45</t>
+        </is>
+      </c>
+      <c r="G178" s="6" t="inlineStr">
+        <is>
+          <t>morel@morel-avocats.fr</t>
+        </is>
+      </c>
+      <c r="H178" s="5" t="inlineStr">
+        <is>
+          <t>www.morel-avocats.fr</t>
+        </is>
+      </c>
+      <c r="I178" s="5" t="inlineStr">
+        <is>
+          <t>Droit pénal, Droit des étrangers</t>
+        </is>
+      </c>
+      <c r="J178" s="4" t="inlineStr">
+        <is>
+          <t>18ème</t>
+        </is>
+      </c>
+      <c r="K178" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L178" s="5" t="inlineStr"/>
+    </row>
+    <row r="179" ht="18" customHeight="1">
+      <c r="A179" s="8" t="n">
+        <v>176</v>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>Avocat Montmartre</t>
+        </is>
+      </c>
+      <c r="C179" s="9" t="inlineStr">
+        <is>
+          <t>8 rue des Abbesses</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="inlineStr">
+        <is>
+          <t>75018</t>
+        </is>
+      </c>
+      <c r="E179" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F179" s="8" t="inlineStr">
+        <is>
+          <t>01 42 52 30 30</t>
+        </is>
+      </c>
+      <c r="G179" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocat-montmartre.fr</t>
+        </is>
+      </c>
+      <c r="H179" s="9" t="inlineStr">
+        <is>
+          <t>www.avocat-montmartre.fr</t>
+        </is>
+      </c>
+      <c r="I179" s="9" t="inlineStr">
+        <is>
+          <t>Droit général, Droit du bail</t>
+        </is>
+      </c>
+      <c r="J179" s="8" t="inlineStr">
+        <is>
+          <t>18ème</t>
+        </is>
+      </c>
+      <c r="K179" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L179" s="9" t="inlineStr"/>
+    </row>
+    <row r="180" ht="18" customHeight="1">
+      <c r="A180" s="4" t="n">
+        <v>177</v>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Haddad</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>24 rue de Belleville</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>75019</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F180" s="4" t="inlineStr">
+        <is>
+          <t>01 42 41 10 10</t>
+        </is>
+      </c>
+      <c r="G180" s="6" t="inlineStr">
+        <is>
+          <t>haddad@haddad-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H180" s="5" t="inlineStr">
+        <is>
+          <t>www.haddad-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I180" s="5" t="inlineStr">
+        <is>
+          <t>Droit pénal, Droit de la famille</t>
+        </is>
+      </c>
+      <c r="J180" s="4" t="inlineStr">
+        <is>
+          <t>19ème</t>
+        </is>
+      </c>
+      <c r="K180" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L180" s="5" t="inlineStr"/>
+    </row>
+    <row r="181" ht="18" customHeight="1">
+      <c r="A181" s="8" t="n">
+        <v>178</v>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
+        <is>
+          <t>Avocats Nation Paris</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="inlineStr">
+        <is>
+          <t>8 avenue Philippe Auguste</t>
+        </is>
+      </c>
+      <c r="D181" s="8" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="E181" s="9" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F181" s="8" t="inlineStr">
+        <is>
+          <t>01 43 73 70 70</t>
+        </is>
+      </c>
+      <c r="G181" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocats-nation.fr</t>
+        </is>
+      </c>
+      <c r="H181" s="9" t="inlineStr">
+        <is>
+          <t>www.avocats-nation.fr</t>
+        </is>
+      </c>
+      <c r="I181" s="9" t="inlineStr">
+        <is>
+          <t>Droit du travail, Licenciement</t>
+        </is>
+      </c>
+      <c r="J181" s="8" t="inlineStr">
+        <is>
+          <t>11ème</t>
+        </is>
+      </c>
+      <c r="K181" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L181" s="9" t="inlineStr"/>
+    </row>
+    <row r="182" ht="18" customHeight="1">
+      <c r="A182" s="4" t="n">
+        <v>179</v>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Aubert Versailles</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>9 rue Carnot</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>78000</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>Versailles</t>
+        </is>
+      </c>
+      <c r="F182" s="4" t="inlineStr">
+        <is>
+          <t>01 39 50 15 15</t>
+        </is>
+      </c>
+      <c r="G182" s="6" t="inlineStr">
+        <is>
+          <t>aubert@aubert-avocat78.fr</t>
+        </is>
+      </c>
+      <c r="H182" s="5" t="inlineStr">
+        <is>
+          <t>www.aubert-avocat78.fr</t>
+        </is>
+      </c>
+      <c r="I182" s="5" t="inlineStr">
+        <is>
+          <t>Droit immobilier, Droit de la famille</t>
+        </is>
+      </c>
+      <c r="J182" s="4" t="inlineStr">
+        <is>
+          <t>Versailles</t>
+        </is>
+      </c>
+      <c r="K182" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L182" s="5" t="inlineStr"/>
+    </row>
+    <row r="183" ht="18" customHeight="1">
+      <c r="A183" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="B183" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Delorme Versailles</t>
+        </is>
+      </c>
+      <c r="C183" s="9" t="inlineStr">
+        <is>
+          <t>14 rue de la Paroisse</t>
+        </is>
+      </c>
+      <c r="D183" s="8" t="inlineStr">
+        <is>
+          <t>78000</t>
+        </is>
+      </c>
+      <c r="E183" s="9" t="inlineStr">
+        <is>
+          <t>Versailles</t>
+        </is>
+      </c>
+      <c r="F183" s="8" t="inlineStr">
+        <is>
+          <t>01 39 53 45 45</t>
+        </is>
+      </c>
+      <c r="G183" s="6" t="inlineStr">
+        <is>
+          <t>delorme@delorme-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H183" s="9" t="inlineStr">
+        <is>
+          <t>www.delorme-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I183" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Droit social</t>
+        </is>
+      </c>
+      <c r="J183" s="8" t="inlineStr">
+        <is>
+          <t>Versailles</t>
+        </is>
+      </c>
+      <c r="K183" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L183" s="9" t="inlineStr"/>
+    </row>
+    <row r="184" ht="18" customHeight="1">
+      <c r="A184" s="4" t="n">
+        <v>181</v>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>Avocat Saint-Denis</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>18 rue de la République</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>93200</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>Saint-Denis</t>
+        </is>
+      </c>
+      <c r="F184" s="4" t="inlineStr">
+        <is>
+          <t>01 48 09 40 40</t>
+        </is>
+      </c>
+      <c r="G184" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocat-saint-denis.fr</t>
+        </is>
+      </c>
+      <c r="H184" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-saint-denis.fr</t>
+        </is>
+      </c>
+      <c r="I184" s="5" t="inlineStr">
+        <is>
+          <t>Droit pénal, Droit des étrangers</t>
+        </is>
+      </c>
+      <c r="J184" s="4" t="inlineStr">
+        <is>
+          <t>Saint-Denis</t>
+        </is>
+      </c>
+      <c r="K184" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L184" s="5" t="inlineStr"/>
+    </row>
+    <row r="185" ht="18" customHeight="1">
+      <c r="A185" s="8" t="n">
+        <v>182</v>
+      </c>
+      <c r="B185" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Menut Montreuil</t>
+        </is>
+      </c>
+      <c r="C185" s="9" t="inlineStr">
+        <is>
+          <t>12 rue de Paris</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="inlineStr">
+        <is>
+          <t>93100</t>
+        </is>
+      </c>
+      <c r="E185" s="9" t="inlineStr">
+        <is>
+          <t>Montreuil</t>
+        </is>
+      </c>
+      <c r="F185" s="8" t="inlineStr">
+        <is>
+          <t>01 48 70 30 30</t>
+        </is>
+      </c>
+      <c r="G185" s="6" t="inlineStr">
+        <is>
+          <t>menut@menut-avocat.fr</t>
+        </is>
+      </c>
+      <c r="H185" s="9" t="inlineStr">
+        <is>
+          <t>www.menut-avocat.fr</t>
+        </is>
+      </c>
+      <c r="I185" s="9" t="inlineStr">
+        <is>
+          <t>Droit social, Droit des locataires</t>
+        </is>
+      </c>
+      <c r="J185" s="8" t="inlineStr">
+        <is>
+          <t>Montreuil</t>
+        </is>
+      </c>
+      <c r="K185" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L185" s="9" t="inlineStr"/>
+    </row>
+    <row r="186" ht="18" customHeight="1">
+      <c r="A186" s="4" t="n">
+        <v>183</v>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Avocats Vincennes</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>5 avenue de Paris</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>94300</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>Vincennes</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t>01 43 28 20 20</t>
+        </is>
+      </c>
+      <c r="G186" s="6" t="inlineStr">
+        <is>
+          <t>contact@avocat-vincennes.fr</t>
+        </is>
+      </c>
+      <c r="H186" s="5" t="inlineStr">
+        <is>
+          <t>www.avocat-vincennes.fr</t>
+        </is>
+      </c>
+      <c r="I186" s="5" t="inlineStr">
+        <is>
+          <t>Droit de la famille, Droit immobilier</t>
+        </is>
+      </c>
+      <c r="J186" s="4" t="inlineStr">
+        <is>
+          <t>Vincennes</t>
+        </is>
+      </c>
+      <c r="K186" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L186" s="5" t="inlineStr"/>
+    </row>
+    <row r="187" ht="18" customHeight="1">
+      <c r="A187" s="8" t="n">
+        <v>184</v>
+      </c>
+      <c r="B187" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Roche Issy</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="inlineStr">
+        <is>
+          <t>22 rue Ernest Renan</t>
+        </is>
+      </c>
+      <c r="D187" s="8" t="inlineStr">
+        <is>
+          <t>92130</t>
+        </is>
+      </c>
+      <c r="E187" s="9" t="inlineStr">
+        <is>
+          <t>Issy-les-Moulineaux</t>
+        </is>
+      </c>
+      <c r="F187" s="8" t="inlineStr">
+        <is>
+          <t>01 41 23 50 50</t>
+        </is>
+      </c>
+      <c r="G187" s="6" t="inlineStr">
+        <is>
+          <t>roche@roche-avocat92.fr</t>
+        </is>
+      </c>
+      <c r="H187" s="9" t="inlineStr">
+        <is>
+          <t>www.roche-avocat92.fr</t>
+        </is>
+      </c>
+      <c r="I187" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Droit social</t>
+        </is>
+      </c>
+      <c r="J187" s="8" t="inlineStr">
+        <is>
+          <t>Issy</t>
+        </is>
+      </c>
+      <c r="K187" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L187" s="9" t="inlineStr"/>
+    </row>
+    <row r="188" ht="18" customHeight="1">
+      <c r="A188" s="4" t="n">
+        <v>185</v>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>Cabinet Simon Levallois</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>33 rue Louis Rouquier</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>92300</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>Levallois-Perret</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="inlineStr">
+        <is>
+          <t>01 47 59 15 15</t>
+        </is>
+      </c>
+      <c r="G188" s="6" t="inlineStr">
+        <is>
+          <t>simon@simon-avocat92.fr</t>
+        </is>
+      </c>
+      <c r="H188" s="5" t="inlineStr">
+        <is>
+          <t>www.simon-avocat92.fr</t>
+        </is>
+      </c>
+      <c r="I188" s="5" t="inlineStr">
+        <is>
+          <t>Droit commercial, Baux commerciaux</t>
+        </is>
+      </c>
+      <c r="J188" s="4" t="inlineStr">
+        <is>
+          <t>Levallois</t>
+        </is>
+      </c>
+      <c r="K188" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L188" s="5" t="inlineStr"/>
+    </row>
+    <row r="189" ht="18" customHeight="1">
+      <c r="A189" s="8" t="n">
+        <v>186</v>
+      </c>
+      <c r="B189" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Martin Nanterre</t>
+        </is>
+      </c>
+      <c r="C189" s="9" t="inlineStr">
+        <is>
+          <t>15 avenue Pablo Picasso</t>
+        </is>
+      </c>
+      <c r="D189" s="8" t="inlineStr">
+        <is>
+          <t>92000</t>
+        </is>
+      </c>
+      <c r="E189" s="9" t="inlineStr">
+        <is>
+          <t>Nanterre</t>
+        </is>
+      </c>
+      <c r="F189" s="8" t="inlineStr">
+        <is>
+          <t>01 47 21 80 80</t>
+        </is>
+      </c>
+      <c r="G189" s="6" t="inlineStr">
+        <is>
+          <t>martin@martin-avocat-nanterre.fr</t>
+        </is>
+      </c>
+      <c r="H189" s="9" t="inlineStr">
+        <is>
+          <t>www.martin-avocat-nanterre.fr</t>
+        </is>
+      </c>
+      <c r="I189" s="9" t="inlineStr">
+        <is>
+          <t>Droit des affaires, Droit du travail</t>
+        </is>
+      </c>
+      <c r="J189" s="8" t="inlineStr">
+        <is>
+          <t>Nanterre</t>
+        </is>
+      </c>
+      <c r="K189" s="7" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="L189" s="9" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:L123"/>
+  <autoFilter ref="A3:L189"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>

</xml_diff>